<commit_message>
Fix three major homepage visual issues: stats, lifecycle wheel, and form
- lifecycle-wheel parser: change output from <ul><li> to <p><a> pairs to
  match the block decorator's expected content model
- columns-media parser: add stat number extraction from
  .paragraph--type--simple-stat elements (7M+, 315M+, 1K+, 24/7)
- import-homepage: wire lifecycle-wheel and form parsers, update section
  definitions so each section uses the correct block parser

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-homepage.report.xlsx
+++ b/tools/importer/reports/import-homepage.report.xlsx
@@ -40,7 +40,7 @@
     <t>index.report.json</t>
   </si>
   <si>
-    <t>["hero-homepage","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","cards-product","cards-news"]</t>
+    <t>["hero-homepage","columns-media","columns-media","columns-media","columns-media","columns-media","cards-product","cards-news","lifecycle-wheel","form"]</t>
   </si>
   <si>
     <t>index</t>
@@ -52,7 +52,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-03-28T22:23:49.715Z</t>
+    <t>2026-03-30T00:46:46.122Z</t>
   </si>
   <si>
     <t>Cvent | Event Platform for In-person, Virtual, and Hybrid Events &amp; Webinars</t>
@@ -73,7 +73,7 @@
     <t>training-certification</t>
   </si>
   <si>
-    <t>2026-03-28T19:39:53.753Z</t>
+    <t>2026-03-28T22:28:18.683Z</t>
   </si>
   <si>
     <t>Cvent Academy | Cvent</t>
@@ -94,7 +94,7 @@
     <t>company-info</t>
   </si>
   <si>
-    <t>2026-03-28T19:38:42.107Z</t>
+    <t>2026-03-28T22:26:30.336Z</t>
   </si>
   <si>
     <t>Awards and Recognition - Event Management | Cvent</t>
@@ -109,7 +109,7 @@
     <t>en/become-partner</t>
   </si>
   <si>
-    <t>2026-03-28T19:38:56.233Z</t>
+    <t>2026-03-28T22:26:42.882Z</t>
   </si>
   <si>
     <t>Partner Program - Join the Cvent Partner Program | Cvent</t>
@@ -130,7 +130,7 @@
     <t>resource-listing</t>
   </si>
   <si>
-    <t>2026-03-28T19:38:05.603Z</t>
+    <t>2026-03-28T22:27:45.370Z</t>
   </si>
   <si>
     <t>Your Hub for Meetings, Hospitality, and Event Excellence | Cvent Blog</t>
@@ -148,7 +148,7 @@
     <t>en/case-studies</t>
   </si>
   <si>
-    <t>2026-03-28T19:38:11.569Z</t>
+    <t>2026-03-28T22:27:51.514Z</t>
   </si>
   <si>
     <t>Cvent Customer Success Stories &amp; Reviews</t>
@@ -166,7 +166,7 @@
     <t>en/company</t>
   </si>
   <si>
-    <t>2026-03-28T19:38:37.479Z</t>
+    <t>2026-03-28T22:26:22.910Z</t>
   </si>
   <si>
     <t>Company Overview | Cvent</t>
@@ -184,7 +184,7 @@
     <t>contact-demo</t>
   </si>
   <si>
-    <t>2026-03-28T19:39:16.088Z</t>
+    <t>2026-03-29T23:21:04.834Z</t>
   </si>
   <si>
     <t>Contact Us | Cvent</t>
@@ -199,7 +199,7 @@
     <t>en/cvent-certification</t>
   </si>
   <si>
-    <t>2026-03-28T19:40:02.106Z</t>
+    <t>2026-03-28T22:28:27.045Z</t>
   </si>
   <si>
     <t>Cvent Certification | Cvent</t>
@@ -217,7 +217,7 @@
     <t>en/cvent-news-and-press-releases</t>
   </si>
   <si>
-    <t>2026-03-28T19:38:31.447Z</t>
+    <t>2026-03-28T22:28:13.765Z</t>
   </si>
   <si>
     <t>Cvent News &amp; Press Releases | Newsroom | Cvent</t>
@@ -229,7 +229,7 @@
     <t>en/cventiq.report.json</t>
   </si>
   <si>
-    <t>["columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","cards-testimonial","cards-testimonial","cards-testimonial","cards-testimonial","cards-testimonial","cards-testimonial"]</t>
+    <t>["columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","cards-testimonial","cards-testimonial","cards-testimonial","cards-testimonial","cards-testimonial","cards-testimonial","cards-feature"]</t>
   </si>
   <si>
     <t>en/cventiq</t>
@@ -238,7 +238,7 @@
     <t>product-platform</t>
   </si>
   <si>
-    <t>2026-03-28T19:36:17.192Z</t>
+    <t>2026-03-29T22:23:24.548Z</t>
   </si>
   <si>
     <t>CventIQ: AI Solutions for Events</t>
@@ -250,13 +250,13 @@
     <t>en/event-management-software.report.json</t>
   </si>
   <si>
-    <t>["hero-product-form","tabs-integrations","columns-media","cards-testimonial"]</t>
+    <t>["hero-product-form","tabs-integrations","columns-media","cards-testimonial","logo-wall","logo-wall","logo-wall","logo-wall","logo-wall","logo-wall","logo-wall"]</t>
   </si>
   <si>
     <t>en/event-management-software</t>
   </si>
   <si>
-    <t>2026-03-28T19:35:39.612Z</t>
+    <t>2026-03-29T23:22:03.683Z</t>
   </si>
   <si>
     <t>Online Event Management Software | Cvent</t>
@@ -268,28 +268,28 @@
     <t>en/event-types.report.json</t>
   </si>
   <si>
+    <t>en/event-types</t>
+  </si>
+  <si>
+    <t>2026-03-29T22:23:17.222Z</t>
+  </si>
+  <si>
+    <t>404 | Cvent</t>
+  </si>
+  <si>
+    <t>https://www.cvent.com/en/event-types</t>
+  </si>
+  <si>
+    <t>en/management-team.report.json</t>
+  </si>
+  <si>
     <t>[]</t>
   </si>
   <si>
-    <t>en/event-types</t>
-  </si>
-  <si>
-    <t>2026-03-28T19:36:10.048Z</t>
-  </si>
-  <si>
-    <t>404 | Cvent</t>
-  </si>
-  <si>
-    <t>https://www.cvent.com/en/event-types</t>
-  </si>
-  <si>
-    <t>en/management-team.report.json</t>
-  </si>
-  <si>
     <t>en/management-team</t>
   </si>
   <si>
-    <t>2026-03-28T19:38:49.010Z</t>
+    <t>2026-03-28T22:26:37.467Z</t>
   </si>
   <si>
     <t>Management Team | Senior Leadership | Cvent</t>
@@ -307,7 +307,7 @@
     <t>legal</t>
   </si>
   <si>
-    <t>2026-03-28T19:39:27.745Z</t>
+    <t>2026-03-28T22:27:16.161Z</t>
   </si>
   <si>
     <t>Cvent Privacy Policy | Cvent</t>
@@ -322,7 +322,7 @@
     <t>en/product-terms-of-use</t>
   </si>
   <si>
-    <t>2026-03-28T19:39:34.504Z</t>
+    <t>2026-03-28T22:27:21.983Z</t>
   </si>
   <si>
     <t>Terms of Use for Cvent Products | Cvent</t>
@@ -340,7 +340,7 @@
     <t>en/products</t>
   </si>
   <si>
-    <t>2026-03-28T19:36:03.690Z</t>
+    <t>2026-03-29T22:23:10.106Z</t>
   </si>
   <si>
     <t>Events &amp; Venue Management Products | Cvent</t>
@@ -352,13 +352,13 @@
     <t>en/request-demo.report.json</t>
   </si>
   <si>
-    <t>["hero-product-form"]</t>
+    <t>["hero-product-form","cards-testimonial","logo-wall"]</t>
   </si>
   <si>
     <t>en/request-demo</t>
   </si>
   <si>
-    <t>2026-03-28T19:39:09.188Z</t>
+    <t>2026-03-29T23:20:57.801Z</t>
   </si>
   <si>
     <t>Cvent Demo | Cvent</t>
@@ -373,7 +373,7 @@
     <t>en/resources</t>
   </si>
   <si>
-    <t>2026-03-28T19:38:26.017Z</t>
+    <t>2026-03-28T22:28:06.524Z</t>
   </si>
   <si>
     <t>Content Library | Resources | Cvent</t>
@@ -391,7 +391,7 @@
     <t>en/security</t>
   </si>
   <si>
-    <t>2026-03-28T19:39:03.024Z</t>
+    <t>2026-03-28T22:26:49.737Z</t>
   </si>
   <si>
     <t>Event Data Security for Customers | Cvent</t>
@@ -412,7 +412,7 @@
     <t>supplier-venue</t>
   </si>
   <si>
-    <t>2026-03-28T19:37:19.532Z</t>
+    <t>2026-03-28T22:25:41.274Z</t>
   </si>
   <si>
     <t>Supplier and Venue Management Solutions | Cvent</t>
@@ -427,7 +427,7 @@
     <t>en/upcoming-webinars</t>
   </si>
   <si>
-    <t>2026-03-28T19:38:17.968Z</t>
+    <t>2026-03-28T22:28:00.140Z</t>
   </si>
   <si>
     <t>Upcoming Events</t>
@@ -442,7 +442,7 @@
     <t>en/website-terms-use</t>
   </si>
   <si>
-    <t>2026-03-28T19:39:41.775Z</t>
+    <t>2026-03-28T22:27:27.800Z</t>
   </si>
   <si>
     <t>Website Terms of Use | Cvent</t>
@@ -457,7 +457,7 @@
     <t>en/company/legal</t>
   </si>
   <si>
-    <t>2026-03-28T19:39:47.502Z</t>
+    <t>2026-03-28T22:27:33.832Z</t>
   </si>
   <si>
     <t>Cvent Legal</t>
@@ -472,7 +472,7 @@
     <t>en/contact/support</t>
   </si>
   <si>
-    <t>2026-03-28T19:39:22.940Z</t>
+    <t>2026-03-29T23:21:10.656Z</t>
   </si>
   <si>
     <t>Cvent Support</t>
@@ -484,13 +484,13 @@
     <t>en/event-management-software/cvent-integrations.report.json</t>
   </si>
   <si>
-    <t>["hero-product-form","tabs-integrations","columns-media","columns-media","columns-media","columns-media"]</t>
+    <t>["hero-product-form","tabs-integrations","columns-media","columns-media","columns-media","columns-media","columns-media","logo-wall","logo-wall","logo-wall","logo-wall","logo-wall","logo-wall","logo-wall"]</t>
   </si>
   <si>
     <t>en/event-management-software/cvent-integrations</t>
   </si>
   <si>
-    <t>2026-03-28T19:35:45.911Z</t>
+    <t>2026-03-29T22:22:54.126Z</t>
   </si>
   <si>
     <t>Meeting &amp; Events Tools Integration With Cvent</t>
@@ -502,13 +502,13 @@
     <t>en/event-management-software/cvent-pricing.report.json</t>
   </si>
   <si>
-    <t>["cards-testimonial","cards-testimonial","cards-testimonial"]</t>
+    <t>["columns-media","columns-media","cards-testimonial","cards-testimonial","cards-testimonial","cards-feature","form","logo-wall"]</t>
   </si>
   <si>
     <t>en/event-management-software/cvent-pricing</t>
   </si>
   <si>
-    <t>2026-03-28T19:35:54.043Z</t>
+    <t>2026-03-29T22:23:03.109Z</t>
   </si>
   <si>
     <t>Cvent Pricing | Request a Quote</t>
@@ -529,7 +529,7 @@
     <t>product-feature</t>
   </si>
   <si>
-    <t>2026-03-28T19:37:13.608Z</t>
+    <t>2026-03-28T22:24:47.274Z</t>
   </si>
   <si>
     <t>Create Accessible Events with Cvent | Cvent</t>
@@ -547,7 +547,7 @@
     <t>en/event-marketing-management/cvent-essentials</t>
   </si>
   <si>
-    <t>2026-03-28T19:36:50.943Z</t>
+    <t>2026-03-28T22:24:23.084Z</t>
   </si>
   <si>
     <t>Cvent Essentials | Cvent</t>
@@ -565,7 +565,7 @@
     <t>en/event-marketing-management/cvent-supplier-network</t>
   </si>
   <si>
-    <t>2026-03-28T19:37:07.548Z</t>
+    <t>2026-03-28T22:24:39.111Z</t>
   </si>
   <si>
     <t>Free Venue Sourcing Tool | Cvent</t>
@@ -583,7 +583,7 @@
     <t>en/event-marketing-management/event-registration-software</t>
   </si>
   <si>
-    <t>2026-03-28T19:36:28.175Z</t>
+    <t>2026-03-28T22:23:57.919Z</t>
   </si>
   <si>
     <t>Online Event Registration Software | Cvent</t>
@@ -601,7 +601,7 @@
     <t>en/event-marketing-management/mobile-event-apps</t>
   </si>
   <si>
-    <t>2026-03-28T19:36:35.198Z</t>
+    <t>2026-03-28T22:24:07.173Z</t>
   </si>
   <si>
     <t>AI-Powered Event App | Cvent</t>
@@ -619,7 +619,7 @@
     <t>en/event-marketing-management/onarrival-event-check-in-software</t>
   </si>
   <si>
-    <t>2026-03-28T19:36:59.498Z</t>
+    <t>2026-03-28T22:24:31.204Z</t>
   </si>
   <si>
     <t>Onsite Event Check-in and Badging Solutions | Cvent</t>
@@ -637,7 +637,7 @@
     <t>en/event-marketing-management/webinar-platform</t>
   </si>
   <si>
-    <t>2026-03-28T19:36:44.137Z</t>
+    <t>2026-03-28T22:24:15.204Z</t>
   </si>
   <si>
     <t>Best Webinar Platform - Deliver Interactive Webinars | Cvent</t>
@@ -655,7 +655,7 @@
     <t>en/supplier-venue/business-travel-solutions</t>
   </si>
   <si>
-    <t>2026-03-28T19:37:59.258Z</t>
+    <t>2026-03-28T22:26:17.535Z</t>
   </si>
   <si>
     <t>Business Travel Solutions | Cvent</t>
@@ -673,7 +673,7 @@
     <t>en/supplier-venue/group-marketing-solutions</t>
   </si>
   <si>
-    <t>2026-03-28T19:37:27.479Z</t>
+    <t>2026-03-28T22:25:49.378Z</t>
   </si>
   <si>
     <t>Group Marketing Solutions | Increase Visibility &amp; Drive Business | Cvent</t>
@@ -691,7 +691,7 @@
     <t>en/supplier-venue/group-operations-solutions</t>
   </si>
   <si>
-    <t>2026-03-28T19:37:41.089Z</t>
+    <t>2026-03-28T22:26:02.633Z</t>
   </si>
   <si>
     <t>Hotel Operations Management Solutions | Cvent</t>
@@ -706,7 +706,7 @@
     <t>en/supplier-venue/group-sales-solutions</t>
   </si>
   <si>
-    <t>2026-03-28T19:37:35.031Z</t>
+    <t>2026-03-28T22:25:56.435Z</t>
   </si>
   <si>
     <t>Hotel Sales Solutions | Maximize Sales &amp; Streamline Bookings | Cvent</t>
@@ -724,7 +724,7 @@
     <t>en/supplier-venue/hotel-business-intelligence</t>
   </si>
   <si>
-    <t>2026-03-28T19:37:49.586Z</t>
+    <t>2026-03-28T22:26:09.880Z</t>
   </si>
   <si>
     <t>Hotel Business Intelligence Software | Data-Driven Growth | Cvent</t>
@@ -742,7 +742,7 @@
     <t>resource-detail</t>
   </si>
   <si>
-    <t>2026-03-28T19:40:08.779Z</t>
+    <t>2026-03-28T22:27:40.483Z</t>
   </si>
   <si>
     <t>Your Top Event Trends for 2026 | Cvent</t>
@@ -1489,10 +1489,10 @@
         <v>84</v>
       </c>
       <c r="B14" t="s">
+        <v>17</v>
+      </c>
+      <c r="C14" t="s">
         <v>85</v>
-      </c>
-      <c r="C14" t="s">
-        <v>86</v>
       </c>
       <c r="D14" t="s">
         <v>11</v>
@@ -1501,21 +1501,21 @@
         <v>74</v>
       </c>
       <c r="F14" t="s">
+        <v>86</v>
+      </c>
+      <c r="G14" t="s">
         <v>87</v>
       </c>
-      <c r="G14" t="s">
+      <c r="H14" t="s">
         <v>88</v>
-      </c>
-      <c r="H14" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>89</v>
+      </c>
+      <c r="B15" t="s">
         <v>90</v>
-      </c>
-      <c r="B15" t="s">
-        <v>85</v>
       </c>
       <c r="C15" t="s">
         <v>91</v>
@@ -1723,7 +1723,7 @@
         <v>136</v>
       </c>
       <c r="B23" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="C23" t="s">
         <v>137</v>
@@ -1749,7 +1749,7 @@
         <v>141</v>
       </c>
       <c r="B24" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="C24" t="s">
         <v>142</v>
@@ -2191,7 +2191,7 @@
         <v>240</v>
       </c>
       <c r="B41" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="C41" t="s">
         <v>241</v>

</xml_diff>

<commit_message>
Fix lifecycle wheel accordion labels and convert logo wall to block
Lifecycle wheel:
- Add feature name mapping in content freshness transformer to replace
  generic "Explore" link text with descriptive names (e.g. "Venue sourcing",
  "Meeting approval & budgeting") that the scraper misses from JS-rendered
  .inner-category spans
- Update parser to also check .inner-category span as primary source

Logo wall:
- Register existing logo-wall parser in homepage import script
- Add logo-wall block to page template section-4 (was default content)
- Logos now render in centered flex grid via logo-wall block decorator

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-homepage.report.xlsx
+++ b/tools/importer/reports/import-homepage.report.xlsx
@@ -40,7 +40,7 @@
     <t>index.report.json</t>
   </si>
   <si>
-    <t>["hero-homepage","columns-media","columns-media","columns-media","columns-media","columns-media","cards-product","cards-news","lifecycle-wheel","form"]</t>
+    <t>["hero-homepage","columns-media","columns-media","columns-media","columns-media","columns-media","cards-product","cards-news","logo-wall","lifecycle-wheel","form"]</t>
   </si>
   <si>
     <t>index</t>
@@ -52,7 +52,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-03-30T03:21:30.443Z</t>
+    <t>2026-03-30T03:36:49.508Z</t>
   </si>
   <si>
     <t>Cvent | Event Platform for In-person, Virtual, and Hybrid Events &amp; Webinars</t>

</xml_diff>

<commit_message>
Use higher-resolution hero image from source page picture element
Update hero-homepage parser to extract the max_1170w source URL from
<picture><source> elements instead of the smaller 800x600 <img> fallback.
Re-import homepage with the corrected image URL.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-homepage.report.xlsx
+++ b/tools/importer/reports/import-homepage.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="268">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="272">
   <si>
     <t>_reportFile</t>
   </si>
@@ -52,7 +52,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-03-30T05:48:59.636Z</t>
+    <t>2026-03-30T07:38:05.236Z</t>
   </si>
   <si>
     <t>Cvent | Event Platform for In-person, Virtual, and Hybrid Events &amp; Webinars</t>
@@ -64,214 +64,223 @@
     <t>en/academy.report.json</t>
   </si>
   <si>
+    <t>["columns-media","columns-media","cards-feature","cards-quote","cards-quote"]</t>
+  </si>
+  <si>
+    <t>en/academy</t>
+  </si>
+  <si>
+    <t>training-certification</t>
+  </si>
+  <si>
+    <t>2026-03-30T06:55:42.849Z</t>
+  </si>
+  <si>
+    <t>Cvent Academy | Cvent</t>
+  </si>
+  <si>
+    <t>https://www.cvent.com/en/academy</t>
+  </si>
+  <si>
+    <t>en/awards.report.json</t>
+  </si>
+  <si>
+    <t>["columns-media"]</t>
+  </si>
+  <si>
+    <t>en/awards</t>
+  </si>
+  <si>
+    <t>company-info</t>
+  </si>
+  <si>
+    <t>2026-03-30T06:55:11.495Z</t>
+  </si>
+  <si>
+    <t>Awards and Recognition - Event Management | Cvent</t>
+  </si>
+  <si>
+    <t>https://www.cvent.com/en/awards</t>
+  </si>
+  <si>
+    <t>en/become-partner.report.json</t>
+  </si>
+  <si>
+    <t>["columns-media","columns-media","accordion","cards-quote","cards-feature","cards-testimonial","cards-testimonial","cards-testimonial"]</t>
+  </si>
+  <si>
+    <t>en/become-partner</t>
+  </si>
+  <si>
+    <t>2026-03-30T06:55:21.892Z</t>
+  </si>
+  <si>
+    <t>Partner Program - Join the Cvent Partner Program | Cvent</t>
+  </si>
+  <si>
+    <t>https://www.cvent.com/en/become-partner</t>
+  </si>
+  <si>
+    <t>en/blog.report.json</t>
+  </si>
+  <si>
+    <t>["cards-resource","cards-resource","cards-resource","cards-resource","cards-resource"]</t>
+  </si>
+  <si>
+    <t>en/blog</t>
+  </si>
+  <si>
+    <t>resource-listing</t>
+  </si>
+  <si>
+    <t>2026-03-30T06:57:55.995Z</t>
+  </si>
+  <si>
+    <t>Your Hub for Meetings, Hospitality, and Event Excellence | Cvent Blog</t>
+  </si>
+  <si>
+    <t>https://www.cvent.com/en/blog</t>
+  </si>
+  <si>
+    <t>en/case-studies.report.json</t>
+  </si>
+  <si>
+    <t>["cards-resource"]</t>
+  </si>
+  <si>
+    <t>en/case-studies</t>
+  </si>
+  <si>
+    <t>2026-03-30T06:58:02.877Z</t>
+  </si>
+  <si>
+    <t>Cvent Customer Success Stories &amp; Reviews</t>
+  </si>
+  <si>
+    <t>https://www.cvent.com/en/case-studies</t>
+  </si>
+  <si>
+    <t>en/company.report.json</t>
+  </si>
+  <si>
+    <t>["columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","logo-wall","form-standalone"]</t>
+  </si>
+  <si>
+    <t>en/company</t>
+  </si>
+  <si>
+    <t>2026-03-30T06:55:04.590Z</t>
+  </si>
+  <si>
+    <t>Company Overview | Cvent</t>
+  </si>
+  <si>
+    <t>https://www.cvent.com/en/company</t>
+  </si>
+  <si>
+    <t>en/contact-us.report.json</t>
+  </si>
+  <si>
+    <t>en/contact-us</t>
+  </si>
+  <si>
+    <t>contact-demo</t>
+  </si>
+  <si>
+    <t>2026-03-29T23:21:04.834Z</t>
+  </si>
+  <si>
+    <t>Contact Us | Cvent</t>
+  </si>
+  <si>
+    <t>https://www.cvent.com/en/contact-us</t>
+  </si>
+  <si>
+    <t>en/cvent-certification.report.json</t>
+  </si>
+  <si>
+    <t>["columns-media","cards-quote","cards-quote","tabs-horizontal"]</t>
+  </si>
+  <si>
+    <t>en/cvent-certification</t>
+  </si>
+  <si>
+    <t>2026-03-30T06:55:50.843Z</t>
+  </si>
+  <si>
+    <t>Cvent Certification | Cvent</t>
+  </si>
+  <si>
+    <t>https://www.cvent.com/en/cvent-certification</t>
+  </si>
+  <si>
+    <t>en/cvent-news-and-press-releases.report.json</t>
+  </si>
+  <si>
+    <t>["cards-resource","cards-resource"]</t>
+  </si>
+  <si>
+    <t>en/cvent-news-and-press-releases</t>
+  </si>
+  <si>
+    <t>2026-03-30T06:58:23.769Z</t>
+  </si>
+  <si>
+    <t>Cvent News &amp; Press Releases | Newsroom | Cvent</t>
+  </si>
+  <si>
+    <t>https://www.cvent.com/en/cvent-news-and-press-releases</t>
+  </si>
+  <si>
+    <t>en/cventiq.report.json</t>
+  </si>
+  <si>
+    <t>["columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","cards-testimonial","cards-testimonial","cards-testimonial","cards-testimonial","cards-testimonial","cards-testimonial","cards-feature","tabs-horizontal","tabs-horizontal","tabs-horizontal","tabs-horizontal","tabs-horizontal"]</t>
+  </si>
+  <si>
+    <t>en/cventiq</t>
+  </si>
+  <si>
+    <t>product-platform</t>
+  </si>
+  <si>
+    <t>2026-03-30T06:56:42.610Z</t>
+  </si>
+  <si>
+    <t>CventIQ: AI Solutions for Events</t>
+  </si>
+  <si>
+    <t>https://www.cvent.com/en/cventiq</t>
+  </si>
+  <si>
+    <t>en/event-management-software.report.json</t>
+  </si>
+  <si>
+    <t>["hero-product-form","tabs-integrations","columns-media","cards-testimonial","logo-wall","logo-wall","logo-wall","logo-wall","logo-wall","logo-wall","logo-wall"]</t>
+  </si>
+  <si>
+    <t>en/event-management-software</t>
+  </si>
+  <si>
+    <t>2026-03-30T06:56:01.799Z</t>
+  </si>
+  <si>
+    <t>Online Event Management Software | Cvent</t>
+  </si>
+  <si>
+    <t>https://www.cvent.com/en/event-management-software</t>
+  </si>
+  <si>
+    <t>en/event-types.report.json</t>
+  </si>
+  <si>
     <t>["columns-media","columns-media"]</t>
   </si>
   <si>
-    <t>en/academy</t>
-  </si>
-  <si>
-    <t>training-certification</t>
-  </si>
-  <si>
-    <t>2026-03-30T05:20:17.762Z</t>
-  </si>
-  <si>
-    <t>Cvent Academy | Cvent</t>
-  </si>
-  <si>
-    <t>https://www.cvent.com/en/academy</t>
-  </si>
-  <si>
-    <t>en/awards.report.json</t>
-  </si>
-  <si>
-    <t>["columns-media"]</t>
-  </si>
-  <si>
-    <t>en/awards</t>
-  </si>
-  <si>
-    <t>company-info</t>
-  </si>
-  <si>
-    <t>2026-03-30T05:19:50.092Z</t>
-  </si>
-  <si>
-    <t>Awards and Recognition - Event Management | Cvent</t>
-  </si>
-  <si>
-    <t>https://www.cvent.com/en/awards</t>
-  </si>
-  <si>
-    <t>en/become-partner.report.json</t>
-  </si>
-  <si>
-    <t>en/become-partner</t>
-  </si>
-  <si>
-    <t>2026-03-30T05:20:04.194Z</t>
-  </si>
-  <si>
-    <t>Partner Program - Join the Cvent Partner Program | Cvent</t>
-  </si>
-  <si>
-    <t>https://www.cvent.com/en/become-partner</t>
-  </si>
-  <si>
-    <t>en/blog.report.json</t>
-  </si>
-  <si>
-    <t>["cards-resource","cards-resource","cards-resource","cards-resource","cards-resource"]</t>
-  </si>
-  <si>
-    <t>en/blog</t>
-  </si>
-  <si>
-    <t>resource-listing</t>
-  </si>
-  <si>
-    <t>2026-03-28T22:27:45.370Z</t>
-  </si>
-  <si>
-    <t>Your Hub for Meetings, Hospitality, and Event Excellence | Cvent Blog</t>
-  </si>
-  <si>
-    <t>https://www.cvent.com/en/blog</t>
-  </si>
-  <si>
-    <t>en/case-studies.report.json</t>
-  </si>
-  <si>
-    <t>["cards-resource"]</t>
-  </si>
-  <si>
-    <t>en/case-studies</t>
-  </si>
-  <si>
-    <t>2026-03-28T22:27:51.514Z</t>
-  </si>
-  <si>
-    <t>Cvent Customer Success Stories &amp; Reviews</t>
-  </si>
-  <si>
-    <t>https://www.cvent.com/en/case-studies</t>
-  </si>
-  <si>
-    <t>en/company.report.json</t>
-  </si>
-  <si>
-    <t>["columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media"]</t>
-  </si>
-  <si>
-    <t>en/company</t>
-  </si>
-  <si>
-    <t>2026-03-30T05:19:44.050Z</t>
-  </si>
-  <si>
-    <t>Company Overview | Cvent</t>
-  </si>
-  <si>
-    <t>https://www.cvent.com/en/company</t>
-  </si>
-  <si>
-    <t>en/contact-us.report.json</t>
-  </si>
-  <si>
-    <t>en/contact-us</t>
-  </si>
-  <si>
-    <t>contact-demo</t>
-  </si>
-  <si>
-    <t>2026-03-29T23:21:04.834Z</t>
-  </si>
-  <si>
-    <t>Contact Us | Cvent</t>
-  </si>
-  <si>
-    <t>https://www.cvent.com/en/contact-us</t>
-  </si>
-  <si>
-    <t>en/cvent-certification.report.json</t>
-  </si>
-  <si>
-    <t>en/cvent-certification</t>
-  </si>
-  <si>
-    <t>2026-03-30T05:20:25.735Z</t>
-  </si>
-  <si>
-    <t>Cvent Certification | Cvent</t>
-  </si>
-  <si>
-    <t>https://www.cvent.com/en/cvent-certification</t>
-  </si>
-  <si>
-    <t>en/cvent-news-and-press-releases.report.json</t>
-  </si>
-  <si>
-    <t>["cards-resource","cards-resource"]</t>
-  </si>
-  <si>
-    <t>en/cvent-news-and-press-releases</t>
-  </si>
-  <si>
-    <t>2026-03-28T22:28:13.765Z</t>
-  </si>
-  <si>
-    <t>Cvent News &amp; Press Releases | Newsroom | Cvent</t>
-  </si>
-  <si>
-    <t>https://www.cvent.com/en/cvent-news-and-press-releases</t>
-  </si>
-  <si>
-    <t>en/cventiq.report.json</t>
-  </si>
-  <si>
-    <t>["columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","cards-testimonial","cards-testimonial","cards-testimonial","cards-testimonial","cards-testimonial","cards-testimonial","cards-feature"]</t>
-  </si>
-  <si>
-    <t>en/cventiq</t>
-  </si>
-  <si>
-    <t>product-platform</t>
-  </si>
-  <si>
-    <t>2026-03-29T22:23:24.548Z</t>
-  </si>
-  <si>
-    <t>CventIQ: AI Solutions for Events</t>
-  </si>
-  <si>
-    <t>https://www.cvent.com/en/cventiq</t>
-  </si>
-  <si>
-    <t>en/event-management-software.report.json</t>
-  </si>
-  <si>
-    <t>["hero-product-form","tabs-integrations","columns-media","cards-testimonial","logo-wall","logo-wall","logo-wall","logo-wall","logo-wall","logo-wall","logo-wall"]</t>
-  </si>
-  <si>
-    <t>en/event-management-software</t>
-  </si>
-  <si>
-    <t>2026-03-29T23:22:03.683Z</t>
-  </si>
-  <si>
-    <t>Online Event Management Software | Cvent</t>
-  </si>
-  <si>
-    <t>https://www.cvent.com/en/event-management-software</t>
-  </si>
-  <si>
-    <t>en/event-types.report.json</t>
-  </si>
-  <si>
     <t>en/event-types</t>
   </si>
   <si>
-    <t>2026-03-29T22:23:17.222Z</t>
+    <t>2026-03-30T06:56:33.111Z</t>
   </si>
   <si>
     <t>404 | Cvent</t>
@@ -289,7 +298,7 @@
     <t>en/management-team</t>
   </si>
   <si>
-    <t>2026-03-30T05:19:56.578Z</t>
+    <t>2026-03-30T06:55:16.391Z</t>
   </si>
   <si>
     <t>Management Team | Senior Leadership | Cvent</t>
@@ -334,13 +343,13 @@
     <t>en/products.report.json</t>
   </si>
   <si>
-    <t>["hero-product-form","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media"]</t>
+    <t>["hero-product-form","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","tabs-horizontal"]</t>
   </si>
   <si>
     <t>en/products</t>
   </si>
   <si>
-    <t>2026-03-29T22:23:10.106Z</t>
+    <t>2026-03-30T06:56:24.487Z</t>
   </si>
   <si>
     <t>Events &amp; Venue Management Products | Cvent</t>
@@ -370,10 +379,13 @@
     <t>en/resources.report.json</t>
   </si>
   <si>
+    <t>["cards-resource","cards-resource","form"]</t>
+  </si>
+  <si>
     <t>en/resources</t>
   </si>
   <si>
-    <t>2026-03-28T22:28:06.524Z</t>
+    <t>2026-03-30T06:58:18.775Z</t>
   </si>
   <si>
     <t>Content Library | Resources | Cvent</t>
@@ -385,13 +397,13 @@
     <t>en/security.report.json</t>
   </si>
   <si>
-    <t>["columns-media","columns-media","columns-media","columns-media","columns-media","columns-media"]</t>
+    <t>["columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","logo-wall","accordion","form-standalone"]</t>
   </si>
   <si>
     <t>en/security</t>
   </si>
   <si>
-    <t>2026-03-30T05:20:12.204Z</t>
+    <t>2026-03-30T06:55:29.947Z</t>
   </si>
   <si>
     <t>Event Data Security for Customers | Cvent</t>
@@ -427,7 +439,7 @@
     <t>en/upcoming-webinars</t>
   </si>
   <si>
-    <t>2026-03-28T22:28:00.140Z</t>
+    <t>2026-03-30T06:58:11.782Z</t>
   </si>
   <si>
     <t>Upcoming Events</t>
@@ -553,13 +565,13 @@
     <t>en/event-management-software/cvent-integrations.report.json</t>
   </si>
   <si>
-    <t>["hero-product-form","tabs-integrations","columns-media","columns-media","columns-media","columns-media","columns-media","logo-wall","logo-wall","logo-wall","logo-wall","logo-wall","logo-wall","logo-wall"]</t>
+    <t>["hero-product-form","tabs-integrations","columns-media","columns-media","columns-media","columns-media","columns-media","logo-wall","logo-wall","logo-wall","logo-wall","logo-wall","logo-wall","logo-wall","tabs-horizontal"]</t>
   </si>
   <si>
     <t>en/event-management-software/cvent-integrations</t>
   </si>
   <si>
-    <t>2026-03-29T22:22:54.126Z</t>
+    <t>2026-03-30T06:56:09.712Z</t>
   </si>
   <si>
     <t>Meeting &amp; Events Tools Integration With Cvent</t>
@@ -577,7 +589,7 @@
     <t>en/event-management-software/cvent-pricing</t>
   </si>
   <si>
-    <t>2026-03-29T22:23:03.109Z</t>
+    <t>2026-03-30T06:56:18.277Z</t>
   </si>
   <si>
     <t>Cvent Pricing | Request a Quote</t>
@@ -598,7 +610,7 @@
     <t>product-feature</t>
   </si>
   <si>
-    <t>2026-03-30T05:15:59.373Z</t>
+    <t>2026-03-30T06:57:40.500Z</t>
   </si>
   <si>
     <t>Create Accessible Events with Cvent | Cvent</t>
@@ -616,7 +628,7 @@
     <t>en/event-marketing-management/cvent-essentials</t>
   </si>
   <si>
-    <t>2026-03-30T05:15:32.605Z</t>
+    <t>2026-03-30T06:57:17.315Z</t>
   </si>
   <si>
     <t>Cvent Essentials | Cvent</t>
@@ -631,7 +643,7 @@
     <t>en/event-marketing-management/cvent-supplier-network</t>
   </si>
   <si>
-    <t>2026-03-30T05:15:51.735Z</t>
+    <t>2026-03-30T06:57:33.331Z</t>
   </si>
   <si>
     <t>Free Venue Sourcing Tool | Cvent</t>
@@ -649,7 +661,7 @@
     <t>en/event-marketing-management/event-registration-software</t>
   </si>
   <si>
-    <t>2026-03-30T05:15:07.561Z</t>
+    <t>2026-03-30T06:56:56.606Z</t>
   </si>
   <si>
     <t>Online Event Registration Software | Cvent</t>
@@ -661,13 +673,13 @@
     <t>en/event-marketing-management/mobile-event-apps.report.json</t>
   </si>
   <si>
-    <t>["hero-product-form","cards-feature","columns-media","columns-media","columns-media","columns-media","columns-media"]</t>
+    <t>["hero-product-form","cards-feature","columns-media","columns-media","columns-media","columns-media","columns-media","accordion"]</t>
   </si>
   <si>
     <t>en/event-marketing-management/mobile-event-apps</t>
   </si>
   <si>
-    <t>2026-03-30T05:15:16.368Z</t>
+    <t>2026-03-30T06:57:04.046Z</t>
   </si>
   <si>
     <t>AI-Powered Event App | Cvent</t>
@@ -685,7 +697,7 @@
     <t>en/event-marketing-management/onarrival-event-check-in-software</t>
   </si>
   <si>
-    <t>2026-03-30T05:15:43.344Z</t>
+    <t>2026-03-30T06:57:26.281Z</t>
   </si>
   <si>
     <t>Onsite Event Check-in and Badging Solutions | Cvent</t>
@@ -703,7 +715,7 @@
     <t>en/event-marketing-management/webinar-platform</t>
   </si>
   <si>
-    <t>2026-03-30T05:15:26.102Z</t>
+    <t>2026-03-30T06:57:10.518Z</t>
   </si>
   <si>
     <t>Best Webinar Platform - Deliver Interactive Webinars | Cvent</t>
@@ -808,7 +820,7 @@
     <t>resource-detail</t>
   </si>
   <si>
-    <t>2026-03-28T22:27:40.483Z</t>
+    <t>2026-03-30T06:58:31.566Z</t>
   </si>
   <si>
     <t>Your Top Event Trends for 2026 | Cvent</t>
@@ -1321,10 +1333,10 @@
         <v>30</v>
       </c>
       <c r="B5" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="C5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D5" t="s">
         <v>11</v>
@@ -1333,76 +1345,76 @@
         <v>26</v>
       </c>
       <c r="F5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D6" t="s">
         <v>11</v>
       </c>
       <c r="E6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D7" t="s">
         <v>11</v>
       </c>
       <c r="E7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="H7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C8" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D8" t="s">
         <v>11</v>
@@ -1411,50 +1423,50 @@
         <v>26</v>
       </c>
       <c r="F8" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G8" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H8" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B9" t="s">
         <v>24</v>
       </c>
       <c r="C9" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D9" t="s">
         <v>11</v>
       </c>
       <c r="E9" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G9" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H9" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B10" t="s">
-        <v>24</v>
+        <v>62</v>
       </c>
       <c r="C10" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D10" t="s">
         <v>11</v>
@@ -1463,128 +1475,128 @@
         <v>19</v>
       </c>
       <c r="F10" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="G10" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="H10" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B11" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C11" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D11" t="s">
         <v>11</v>
       </c>
       <c r="E11" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F11" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G11" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="H11" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C12" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D12" t="s">
         <v>11</v>
       </c>
       <c r="E12" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F12" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="G12" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H12" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B13" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C13" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D13" t="s">
         <v>11</v>
       </c>
       <c r="E13" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F13" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="G13" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="H13" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B14" t="s">
-        <v>17</v>
+        <v>87</v>
       </c>
       <c r="C14" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="D14" t="s">
         <v>11</v>
       </c>
       <c r="E14" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F14" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="G14" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="H14" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="B15" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="C15" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="D15" t="s">
         <v>11</v>
@@ -1593,154 +1605,154 @@
         <v>26</v>
       </c>
       <c r="F15" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="G15" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="H15" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="B16" t="s">
         <v>24</v>
       </c>
       <c r="C16" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="D16" t="s">
         <v>11</v>
       </c>
       <c r="E16" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="F16" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="G16" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="H16" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="B17" t="s">
         <v>24</v>
       </c>
       <c r="C17" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="D17" t="s">
         <v>11</v>
       </c>
       <c r="E17" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="F17" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="G17" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="H17" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="B18" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="C18" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="D18" t="s">
         <v>11</v>
       </c>
       <c r="E18" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F18" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="G18" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="H18" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="B19" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="C19" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="D19" t="s">
         <v>11</v>
       </c>
       <c r="E19" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F19" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="G19" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="H19" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="B20" t="s">
-        <v>66</v>
+        <v>122</v>
       </c>
       <c r="C20" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="D20" t="s">
         <v>11</v>
       </c>
       <c r="E20" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F20" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="G20" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="H20" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="B21" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="C21" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="D21" t="s">
         <v>11</v>
@@ -1749,663 +1761,663 @@
         <v>26</v>
       </c>
       <c r="F21" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="G21" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="H21" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="B22" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="C22" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="D22" t="s">
         <v>11</v>
       </c>
       <c r="E22" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="F22" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="G22" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="H22" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B23" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="C23" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="D23" t="s">
         <v>11</v>
       </c>
       <c r="E23" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F23" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="G23" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="H23" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="B24" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="C24" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="D24" t="s">
         <v>11</v>
       </c>
       <c r="E24" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="F24" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="G24" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="H24" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B25" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="C25" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="D25" t="s">
         <v>11</v>
       </c>
       <c r="E25" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="F25" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="G25" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="H25" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="B26" t="s">
+        <v>157</v>
+      </c>
+      <c r="C26" t="s">
+        <v>158</v>
+      </c>
+      <c r="D26" t="s">
+        <v>11</v>
+      </c>
+      <c r="E26" t="s">
         <v>153</v>
       </c>
-      <c r="C26" t="s">
-        <v>154</v>
-      </c>
-      <c r="D26" t="s">
-        <v>11</v>
-      </c>
-      <c r="E26" t="s">
-        <v>149</v>
-      </c>
       <c r="F26" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="G26" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="H26" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="B27" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="C27" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="D27" t="s">
         <v>11</v>
       </c>
       <c r="E27" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="F27" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="G27" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="H27" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="B28" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="C28" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="D28" t="s">
         <v>11</v>
       </c>
       <c r="E28" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="F28" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="G28" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="H28" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="B29" t="s">
+        <v>157</v>
+      </c>
+      <c r="C29" t="s">
+        <v>171</v>
+      </c>
+      <c r="D29" t="s">
+        <v>11</v>
+      </c>
+      <c r="E29" t="s">
         <v>153</v>
       </c>
-      <c r="C29" t="s">
-        <v>167</v>
-      </c>
-      <c r="D29" t="s">
-        <v>11</v>
-      </c>
-      <c r="E29" t="s">
-        <v>149</v>
-      </c>
       <c r="F29" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="G29" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="H29" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="B30" t="s">
         <v>24</v>
       </c>
       <c r="C30" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="D30" t="s">
         <v>11</v>
       </c>
       <c r="E30" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="F30" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="G30" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="H30" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="B31" t="s">
-        <v>17</v>
+        <v>87</v>
       </c>
       <c r="C31" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="D31" t="s">
         <v>11</v>
       </c>
       <c r="E31" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F31" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="G31" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="H31" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="B32" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="C32" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="D32" t="s">
         <v>11</v>
       </c>
       <c r="E32" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F32" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="G32" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="H32" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="B33" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="C33" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="D33" t="s">
         <v>11</v>
       </c>
       <c r="E33" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F33" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="G33" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="H33" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="B34" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="C34" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="D34" t="s">
         <v>11</v>
       </c>
       <c r="E34" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="F34" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="G34" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="H34" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
+        <v>202</v>
+      </c>
+      <c r="B35" t="s">
+        <v>203</v>
+      </c>
+      <c r="C35" t="s">
+        <v>204</v>
+      </c>
+      <c r="D35" t="s">
+        <v>11</v>
+      </c>
+      <c r="E35" t="s">
         <v>198</v>
       </c>
-      <c r="B35" t="s">
-        <v>199</v>
-      </c>
-      <c r="C35" t="s">
-        <v>200</v>
-      </c>
-      <c r="D35" t="s">
-        <v>11</v>
-      </c>
-      <c r="E35" t="s">
-        <v>194</v>
-      </c>
       <c r="F35" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="G35" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="H35" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="B36" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="C36" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="D36" t="s">
         <v>11</v>
       </c>
       <c r="E36" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="F36" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="G36" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="H36" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="B37" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="C37" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="D37" t="s">
         <v>11</v>
       </c>
       <c r="E37" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="F37" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="G37" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="H37" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="B38" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="C38" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="D38" t="s">
         <v>11</v>
       </c>
       <c r="E38" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="F38" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="G38" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="H38" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="B39" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="C39" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="D39" t="s">
         <v>11</v>
       </c>
       <c r="E39" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="F39" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="G39" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="H39" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="B40" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="C40" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="D40" t="s">
         <v>11</v>
       </c>
       <c r="E40" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="F40" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="G40" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="H40" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="B41" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="C41" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="D41" t="s">
         <v>11</v>
       </c>
       <c r="E41" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="F41" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="G41" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="H41" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="B42" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="C42" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="D42" t="s">
         <v>11</v>
       </c>
       <c r="E42" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="F42" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="G42" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="H42" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="B43" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="C43" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="D43" t="s">
         <v>11</v>
       </c>
       <c r="E43" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="F43" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="G43" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="H43" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="B44" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="C44" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="D44" t="s">
         <v>11</v>
       </c>
       <c r="E44" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="F44" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="G44" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="H44" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="B45" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="C45" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="D45" t="s">
         <v>11</v>
       </c>
       <c r="E45" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="F45" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="G45" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="H45" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="B46" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="C46" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="D46" t="s">
         <v>11</v>
       </c>
       <c r="E46" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="F46" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="G46" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="H46" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
   </sheetData>

</xml_diff>